<commit_message>
Update soccer trades 2026-08-10 15:03:09 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V2"/>
+  <dimension ref="A1:V3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,110 +531,222 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-10 17:02:29 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V3"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>5.00692</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.7012</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786377754</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>7.139993</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,110 +643,334 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-10 19:02:44 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V5"/>
+  <dimension ref="A1:V6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -586,7 +586,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +616,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786385932</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +626,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786377754</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -755,12 +755,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -770,22 +770,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>5.00692</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.7012</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786377751</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +850,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>7.139993</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,110 +867,222 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 00:02:34 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V6"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,12 +546,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.1562</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -561,7 +561,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786395562</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>6.464</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,22 +658,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -728,7 +728,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786385932</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -738,7 +738,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +755,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786377754</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -867,12 +867,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -882,22 +882,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>5.00692</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.7012</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786377751</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -962,7 +962,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>7.139993</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -979,110 +979,222 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="O7" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 04:02:53 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V7"/>
+  <dimension ref="A1:V8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,102 +531,94 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>1.125</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>1.01</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>1.1562</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>L19052123</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>SUCCESS</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786412670</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,12 +635,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -658,12 +650,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.1562</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -673,7 +665,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -683,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -728,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786395562</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>6.464</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -755,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -770,22 +762,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -810,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -840,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786385932</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -850,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,7 +859,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -952,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786377754</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -979,12 +971,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -994,22 +986,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>5.00692</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.7012</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1034,7 +1026,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1064,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786377751</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1074,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>7.139993</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1091,110 +1083,222 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="O8" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 07:03:15 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V8"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,17 +542,17 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>90.44268</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.8363</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786412670</t>
+          <t>1786430935</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>108.152682</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.1562</t>
+          <t>1.5525</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Deportes Tolima vs Independiente del Valle</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente del Valle</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051703</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786430206</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>1.809955</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,62 +747,54 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.125</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -832,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786412670</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -842,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +851,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,22 +866,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.1562</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786395562</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>6.464</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +963,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -986,22 +978,22 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1026,7 +1018,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1056,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786385932</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1066,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1083,12 +1075,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1098,22 +1090,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>5.00692</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.7012</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1138,7 +1130,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1168,7 +1160,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786377754</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1178,7 +1170,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>7.139993</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1195,110 +1187,334 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 09:02:45 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:V14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,7 +531,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -542,12 +542,12 @@
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>90.44268</t>
+          <t>2.74998</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.8363</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -608,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786430935</t>
+          <t>1786438265</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -618,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>108.152682</t>
+          <t>3.709922</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,12 +635,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -650,22 +650,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>19.42</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Deportes Tolima vs Independiente del Valle</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Independiente del Valle</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19051703</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786430206</t>
+          <t>1786436520</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>1.809955</t>
+          <t>34.070175</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,23 +755,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -794,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -824,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786412670</t>
+          <t>1786435951</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>3.561404</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -866,12 +874,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.1562</t>
+          <t>1.1687</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -881,7 +889,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -891,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786435593</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>266.666667</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,27 +971,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>90.44268</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.8363</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -991,31 +995,27 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786430935</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1058,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>108.152682</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,12 +1075,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1090,22 +1090,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.5525</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1115,27 +1115,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Deportes Tolima vs Independiente del Valle</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Independiente del Valle</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19051703</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,17 +1160,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786430206</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>1.809955</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,39 +1187,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.125</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1242,7 +1234,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1272,7 +1264,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786412670</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1282,7 +1274,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1299,7 +1291,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1314,22 +1306,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.1562</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1339,27 +1331,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1384,17 +1376,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786395562</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>6.464</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1411,110 +1403,558 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>1786385932</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>1786377754</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P10" t="inlineStr">
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr">
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="T14" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 10:03:17 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V14"/>
+  <dimension ref="A1:V21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,23 +531,27 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
+          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2.74998</t>
+          <t>10.99999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -555,7 +559,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786438265</t>
+          <t>1786442391</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>3.709922</t>
+          <t>18.9655</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
+          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,19 +651,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>19.42</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -663,11 +667,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786436520</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>34.070175</t>
+          <t>23.809524</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
+          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,31 +755,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>27.83</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.5825</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -787,27 +779,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +824,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786435951</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>3.561404</t>
+          <t>47.776824</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,12 +851,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
+          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -874,12 +866,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>48.99946</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.1687</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -889,7 +881,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Tie</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -899,27 +891,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -944,17 +936,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786435593</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>266.666667</t>
+          <t>181.479481</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,7 +963,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -979,15 +971,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>90.44268</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.8363</t>
+          <t>1.155</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -995,7 +991,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1003,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786430935</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>108.152682</t>
+          <t>12.387097</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,39 +1075,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.415</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1115,27 +1107,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Deportes Tolima vs Independiente del Valle</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Independiente del Valle</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19051703</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1160,7 +1152,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786430206</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1170,7 +1162,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>1.809955</t>
+          <t>24.096386</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1187,7 +1179,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1195,23 +1187,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>121.005</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1219,27 +1219,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1264,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786412670</t>
+          <t>1786440700</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>201.675</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,27 +1291,23 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>2.74998</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.1562</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1319,11 +1315,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
+      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1331,27 +1323,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1376,17 +1368,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786438265</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>3.709922</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1403,12 +1395,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1418,12 +1410,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>19.42</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1433,32 +1425,32 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1488,7 +1480,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786436520</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1498,7 +1490,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>34.070175</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1515,12 +1507,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1530,22 +1522,22 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1570,7 +1562,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1600,7 +1592,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786435951</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1610,7 +1602,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>3.561404</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1627,12 +1619,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1642,22 +1634,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.1687</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1682,7 +1674,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1712,7 +1704,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786435593</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1722,7 +1714,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>266.666667</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1739,39 +1731,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>90.44268</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.8363</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1794,7 +1778,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1824,7 +1808,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786430935</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1834,7 +1818,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>108.152682</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1851,110 +1835,886 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>1.5525</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Deportes Tolima vs Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>L19051703</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>1786430206</t>
+        </is>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>1.809955</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>1.125</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>1786412670</t>
+        </is>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>1.1562</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>L19052123</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>1786395562</t>
+        </is>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>6.464</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>1786385932</t>
+        </is>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1786377754</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G21" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H21" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr">
+      <c r="I21" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr">
+      <c r="J21" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K14" t="inlineStr">
+      <c r="K21" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L14" t="inlineStr">
+      <c r="L21" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M14" t="inlineStr">
+      <c r="M21" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R14" t="inlineStr">
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr">
+      <c r="S21" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="T21" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="U21" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="V21" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 11:03:23 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V21"/>
+  <dimension ref="A1:V29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,12 +531,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
+          <t>0xb3a32bdd398462cad567ce66c61f991efd7fcf97116aadff293947265a593cb1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -546,22 +546,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.99999</t>
+          <t>6.035</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.3912</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -571,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -616,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786442391</t>
+          <t>1786445807</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>18.9655</t>
+          <t>15.42492</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
+          <t>0xe14e1c541902c495d865fcecd4beaa322f341ba7d25fe03284d1ed1752b5d581</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -654,12 +654,12 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.57998</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -675,27 +675,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
@@ -720,17 +720,17 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786445791</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>23.809524</t>
+          <t>4.287401</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
+          <t>0x05ff10b7369e329d09c098dea279a2087aef3f99e7333d016cc17fefdc43ac4d</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,23 +755,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>27.83</t>
+          <t>27.85</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.5825</t>
+          <t>1.575</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -794,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -824,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786445438</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>47.776824</t>
+          <t>48.434783</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,12 +859,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
+          <t>0x2ec5d54c918955931d119282e1be426873e354299fd66bdf880768599903ebee</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -866,22 +874,22 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>48.99946</t>
+          <t>8.8513</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.3938</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -891,27 +899,27 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
@@ -936,17 +944,17 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786445410</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>181.479481</t>
+          <t>22.479492</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -963,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
+          <t>0x3d9a529160e80eb890a16c2893670e9bf2273f2addb5d0a989210dceae52707f</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -971,19 +979,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>46.02996</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.155</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -991,11 +995,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1003,27 +1003,27 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
@@ -1048,17 +1048,17 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786445409</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>12.387097</t>
+          <t>55.125701</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,7 +1075,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
+          <t>0x8e51b7cdf462005f489e66cfca0c7d500669ca43fd2d3996f64b84072d635325</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1086,17 +1086,17 @@
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4.27</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.415</t>
+          <t>1.1013</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -1107,27 +1107,27 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
@@ -1152,17 +1152,17 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786445383</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>24.096386</t>
+          <t>42.17284</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,39 +1179,31 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
+          <t>0x56b9d5cfed219c2b12d04856ee24a476270becbad5defbb7dc7dad60a16a13a9</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>121.005</t>
+          <t>12.76064</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1219,27 +1211,27 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
@@ -1264,17 +1256,17 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786440700</t>
+          <t>1786443421</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>201.675</t>
+          <t>28.919297</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1291,28 +1283,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
+          <t>0x35b58acc470365a2c9a245983b170aeeb2f01a388be1e73823eb3f0e1792d4d0</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.74998</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.1375</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1323,27 +1315,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Platense vs Coquimbo Unido</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Platense</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Coquimbo Unido</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
+          <t>0xb869bcff5be47e69467bcfd6e205de9f4533f12ba3b8f1bb20d9de6a5a8aec91</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052327</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1368,17 +1360,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786438265</t>
+          <t>1786442613</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786572000</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>3.709922</t>
+          <t>10.036364</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1395,12 +1387,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
+          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1410,12 +1402,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>19.42</t>
+          <t>10.99999</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1425,7 +1417,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1435,27 +1427,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1480,17 +1472,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786436520</t>
+          <t>1786442391</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>34.070175</t>
+          <t>18.9655</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1507,7 +1499,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
+          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1515,19 +1507,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1535,11 +1523,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
+      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1547,27 +1531,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1592,17 +1576,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786435951</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>3.561404</t>
+          <t>23.809524</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1619,39 +1603,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
+          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
       <c r="D12" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>27.83</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.1687</t>
+          <t>1.5825</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1659,27 +1635,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1704,17 +1680,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786435593</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>266.666667</t>
+          <t>47.776824</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1731,7 +1707,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1739,15 +1715,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>90.44268</t>
+          <t>48.99946</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.8363</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1755,7 +1735,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H13" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1763,27 +1747,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1808,17 +1792,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786430935</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>108.152682</t>
+          <t>181.479481</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1835,12 +1819,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1850,22 +1834,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.155</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1875,27 +1859,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Deportes Tolima vs Independiente del Valle</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Independiente del Valle</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19051703</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1920,7 +1904,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786430206</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1930,7 +1914,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>1.809955</t>
+          <t>12.387097</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1947,7 +1931,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1958,17 +1942,17 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.415</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1979,27 +1963,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2024,17 +2008,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786412670</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>24.096386</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2051,12 +2035,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2066,12 +2050,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>121.005</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.1562</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -2081,32 +2065,32 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
           <t>Universidad Catolica Santiago</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2136,7 +2120,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786440700</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2146,7 +2130,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>201.675</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2163,27 +2147,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.74998</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2191,34 +2171,30 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr">
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2248,7 +2224,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786438265</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2258,7 +2234,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>3.709922</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2275,12 +2251,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2290,22 +2266,22 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>19.42</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2330,7 +2306,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2360,7 +2336,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786436520</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2370,7 +2346,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>34.070175</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2387,12 +2363,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2402,22 +2378,22 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -2442,7 +2418,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
@@ -2472,7 +2448,7 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786435951</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2482,7 +2458,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>3.561404</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2499,12 +2475,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2514,22 +2490,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.1687</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2554,7 +2530,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2584,7 +2560,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786435593</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2594,7 +2570,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>266.666667</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2611,110 +2587,990 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>90.44268</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1.8363</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>1786430935</t>
+        </is>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>108.152682</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1.5525</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Deportes Tolima vs Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>L19051703</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>1786430206</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>1.809955</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>1.125</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R23" t="inlineStr">
+        <is>
+          <t>1786412670</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1.1562</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>L19052123</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>1786395562</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>6.464</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>1786385932</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1786377754</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U27" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U28" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
+      <c r="G29" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr">
+      <c r="I29" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr">
+      <c r="J29" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K21" t="inlineStr">
+      <c r="K29" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L21" t="inlineStr">
+      <c r="L29" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M21" t="inlineStr">
+      <c r="M29" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr">
+      <c r="S29" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T21" t="inlineStr">
+      <c r="T29" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U21" t="inlineStr">
+      <c r="U29" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V21" t="inlineStr">
+      <c r="V29" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 12:03:16 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V29"/>
+  <dimension ref="A1:V37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,39 +531,31 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xb3a32bdd398462cad567ce66c61f991efd7fcf97116aadff293947265a593cb1</t>
+          <t>0xfe9a509a313ff07389ffbf579a41acd018137e511ac3bf176d2373de751fdb99</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6.035</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.3912</t>
+          <t>1.1462</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -586,7 +578,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -616,7 +608,7 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786445807</t>
+          <t>1786448309</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -626,7 +618,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>15.42492</t>
+          <t>68.376068</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -643,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xe14e1c541902c495d865fcecd4beaa322f341ba7d25fe03284d1ed1752b5d581</t>
+          <t>0x055ed722ad8e1fcb4f4772d6b728782e9d84139fc360e9ede36ff234eccc31e5</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -654,7 +646,7 @@
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>3.57998</t>
+          <t>9.08997</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -720,7 +712,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786445791</t>
+          <t>1786447047</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +722,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>4.287401</t>
+          <t>10.886192</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +739,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x05ff10b7369e329d09c098dea279a2087aef3f99e7333d016cc17fefdc43ac4d</t>
+          <t>0x6f820abf55d5322626469d5a3118ee5f9c3a29d1d3a3a6a566e5b199d600f80e</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,31 +747,23 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>27.85</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.575</t>
+          <t>1.4863</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -787,27 +771,27 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -832,17 +816,17 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786445438</t>
+          <t>1786447020</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>48.434783</t>
+          <t>6.107969</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -859,39 +843,31 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x2ec5d54c918955931d119282e1be426873e354299fd66bdf880768599903ebee</t>
+          <t>0x2b58c8cc2c4a11d63f4809e837d399bdea22a0fe868c2eb6e45b6d908e34bd81</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>8.8513</t>
+          <t>18.67</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.3938</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -914,7 +890,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -944,7 +920,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786445410</t>
+          <t>1786446437</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -954,7 +930,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>22.479492</t>
+          <t>22.359281</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -971,31 +947,39 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x3d9a529160e80eb890a16c2893670e9bf2273f2addb5d0a989210dceae52707f</t>
+          <t>0x9108ebe29dd968cf40c2da378f9f378c80aa47fb35d0f66c34ba20823eac7e31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>46.02996</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.835</t>
+          <t>1.5288</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1018,7 +1002,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1048,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786445409</t>
+          <t>1786446431</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1058,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>55.125701</t>
+          <t>1.891253</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1075,31 +1059,39 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x8e51b7cdf462005f489e66cfca0c7d500669ca43fd2d3996f64b84072d635325</t>
+          <t>0x3e490a020b088d367b2092a71abad1210bb7b27c2b51413d74ae52db826f7a65</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>4.27</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.1013</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1122,7 +1114,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1152,7 +1144,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786445383</t>
+          <t>1786446420</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1162,7 +1154,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>42.17284</t>
+          <t>11.631579</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1179,28 +1171,28 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x56b9d5cfed219c2b12d04856ee24a476270becbad5defbb7dc7dad60a16a13a9</t>
+          <t>0x403efc488fdcf260a44f7bf6f00c26c8886eb1811b8c736b1a20b47ca921c66e</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>12.76064</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.105</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -1226,7 +1218,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
+          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1256,7 +1248,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786443421</t>
+          <t>1786446337</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1266,7 +1258,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>28.919297</t>
+          <t>38.952381</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1283,28 +1275,28 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x35b58acc470365a2c9a245983b170aeeb2f01a388be1e73823eb3f0e1792d4d0</t>
+          <t>0x531f4b82607f405ee467b383cf29c72318f248d39b819f053b24ee23023d1f70</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1.36996</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.1375</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -1315,27 +1307,27 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Platense vs Coquimbo Unido</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Platense</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Coquimbo Unido</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xb869bcff5be47e69467bcfd6e205de9f4533f12ba3b8f1bb20d9de6a5a8aec91</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>L19052327</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
@@ -1360,17 +1352,17 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786442613</t>
+          <t>1786446336</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>1786572000</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>10.036364</t>
+          <t>1.640671</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1387,12 +1379,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
+          <t>0xb3a32bdd398462cad567ce66c61f991efd7fcf97116aadff293947265a593cb1</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1402,22 +1394,22 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.99999</t>
+          <t>6.035</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.3912</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1427,27 +1419,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1472,17 +1464,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786442391</t>
+          <t>1786445807</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>18.9655</t>
+          <t>15.42492</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1499,7 +1491,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
+          <t>0xe14e1c541902c495d865fcecd4beaa322f341ba7d25fe03284d1ed1752b5d581</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1510,12 +1502,12 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>3.57998</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1531,27 +1523,27 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
@@ -1576,17 +1568,17 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786445791</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>23.809524</t>
+          <t>4.287401</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1603,7 +1595,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
+          <t>0x05ff10b7369e329d09c098dea279a2087aef3f99e7333d016cc17fefdc43ac4d</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1611,23 +1603,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>27.83</t>
+          <t>27.85</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.5825</t>
+          <t>1.575</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H12" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1650,7 +1650,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -1680,7 +1680,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786445438</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1690,7 +1690,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>47.776824</t>
+          <t>48.434783</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,12 +1707,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
+          <t>0x2ec5d54c918955931d119282e1be426873e354299fd66bdf880768599903ebee</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1722,22 +1722,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>48.99946</t>
+          <t>8.8513</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.3938</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1747,27 +1747,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1792,17 +1792,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786445410</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>181.479481</t>
+          <t>22.479492</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,7 +1819,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
+          <t>0x3d9a529160e80eb890a16c2893670e9bf2273f2addb5d0a989210dceae52707f</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1827,19 +1827,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>46.02996</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.155</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1847,11 +1843,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1859,27 +1851,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1904,17 +1896,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786445409</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>12.387097</t>
+          <t>55.125701</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1931,7 +1923,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
+          <t>0x8e51b7cdf462005f489e66cfca0c7d500669ca43fd2d3996f64b84072d635325</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1942,17 +1934,17 @@
       <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4.27</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.415</t>
+          <t>1.1013</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G15" t="inlineStr"/>
@@ -1963,27 +1955,27 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
@@ -2008,17 +2000,17 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786445383</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>24.096386</t>
+          <t>42.17284</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2035,39 +2027,31 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
+          <t>0x56b9d5cfed219c2b12d04856ee24a476270becbad5defbb7dc7dad60a16a13a9</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>121.005</t>
+          <t>12.76064</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2075,27 +2059,27 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
@@ -2120,17 +2104,17 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786440700</t>
+          <t>1786443421</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>201.675</t>
+          <t>28.919297</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2147,28 +2131,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
+          <t>0x35b58acc470365a2c9a245983b170aeeb2f01a388be1e73823eb3f0e1792d4d0</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>2.74998</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.1375</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -2179,27 +2163,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Platense vs Coquimbo Unido</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Platense</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Coquimbo Unido</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
+          <t>0xb869bcff5be47e69467bcfd6e205de9f4533f12ba3b8f1bb20d9de6a5a8aec91</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052327</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2224,17 +2208,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786438265</t>
+          <t>1786442613</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786572000</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>3.709922</t>
+          <t>10.036364</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2251,12 +2235,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
+          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2266,12 +2250,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>19.42</t>
+          <t>10.99999</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -2281,7 +2265,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -2291,27 +2275,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2336,17 +2320,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786436520</t>
+          <t>1786442391</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>34.070175</t>
+          <t>18.9655</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2363,7 +2347,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
+          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2371,19 +2355,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -2391,11 +2371,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
+      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2403,27 +2379,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2448,17 +2424,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786435951</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>3.561404</t>
+          <t>23.809524</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2475,39 +2451,31 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
+          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr"/>
       <c r="D20" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>27.83</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.1687</t>
+          <t>1.5825</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2515,27 +2483,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2560,17 +2528,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786435593</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>266.666667</t>
+          <t>47.776824</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2587,7 +2555,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2595,15 +2563,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>90.44268</t>
+          <t>48.99946</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.8363</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2611,7 +2583,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2619,27 +2595,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2664,17 +2640,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786430935</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>108.152682</t>
+          <t>181.479481</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2691,12 +2667,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2706,22 +2682,22 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.155</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2731,27 +2707,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Deportes Tolima vs Independiente del Valle</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Independiente del Valle</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19051703</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2776,7 +2752,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786430206</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2786,7 +2762,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>1.809955</t>
+          <t>12.387097</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2803,7 +2779,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2814,17 +2790,17 @@
       <c r="C23" t="inlineStr"/>
       <c r="D23" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.415</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G23" t="inlineStr"/>
@@ -2835,27 +2811,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2880,17 +2856,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786412670</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>24.096386</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2907,12 +2883,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2922,12 +2898,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>121.005</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.1562</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2937,32 +2913,32 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
           <t>Universidad Catolica Santiago</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2992,7 +2968,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786440700</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -3002,7 +2978,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>201.675</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -3019,27 +2995,23 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>2.74998</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3047,34 +3019,30 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
@@ -3104,7 +3072,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786438265</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3114,7 +3082,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>3.709922</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3131,12 +3099,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3146,22 +3114,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>19.42</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3186,7 +3154,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
@@ -3216,7 +3184,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786436520</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -3226,7 +3194,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>34.070175</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3243,12 +3211,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3258,22 +3226,22 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -3298,7 +3266,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3328,7 +3296,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786435951</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3338,7 +3306,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>3.561404</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3355,12 +3323,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3370,22 +3338,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.1687</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -3410,7 +3378,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3440,7 +3408,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786435593</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3450,7 +3418,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>266.666667</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3467,110 +3435,990 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>90.44268</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>1.8363</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>1786430935</t>
+        </is>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>108.152682</t>
+        </is>
+      </c>
+      <c r="U29" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>1.5525</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Deportes Tolima vs Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>L19051703</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>1786430206</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>1.809955</t>
+        </is>
+      </c>
+      <c r="U30" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1.125</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>1786412670</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="U31" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>1.1562</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>L19052123</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>1786395562</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>6.464</t>
+        </is>
+      </c>
+      <c r="U32" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>1786385932</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T33" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="U33" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>1786377754</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U34" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U35" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U36" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V36" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
+      <c r="F37" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr">
+      <c r="G37" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
+      <c r="H37" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr">
+      <c r="I37" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr">
+      <c r="J37" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr">
+      <c r="K37" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L29" t="inlineStr">
+      <c r="L37" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M29" t="inlineStr">
+      <c r="M37" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P29" t="inlineStr">
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R29" t="inlineStr">
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S29" t="inlineStr">
+      <c r="S37" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr">
+      <c r="T37" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U29" t="inlineStr">
+      <c r="U37" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V29" t="inlineStr">
+      <c r="V37" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 13:02:52 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V37"/>
+  <dimension ref="A1:V39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,28 +531,28 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xfe9a509a313ff07389ffbf579a41acd018137e511ac3bf176d2373de751fdb99</t>
+          <t>0xa43e73fd0eb9b697155001cb7d168e615b053bb2384172434ebb7e2cad4f821b</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4.52999</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.1462</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -563,27 +563,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +608,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786448309</t>
+          <t>1786451158</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>68.376068</t>
+          <t>5.3294</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +635,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0x055ed722ad8e1fcb4f4772d6b728782e9d84139fc360e9ede36ff234eccc31e5</t>
+          <t>0xa379a926c9e1de27f304fc4c2c017caa09967132b53155a53855c3019d081a23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,15 +643,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>9.08997</t>
+          <t>7.17</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.835</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -659,7 +663,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -682,7 +690,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -712,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786447047</t>
+          <t>1786450013</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -722,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>10.886192</t>
+          <t>12.803571</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -739,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0x6f820abf55d5322626469d5a3118ee5f9c3a29d1d3a3a6a566e5b199d600f80e</t>
+          <t>0xfe9a509a313ff07389ffbf579a41acd018137e511ac3bf176d2373de751fdb99</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -750,17 +758,17 @@
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.4863</t>
+          <t>1.1462</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (1)</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -786,7 +794,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -816,7 +824,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786447020</t>
+          <t>1786448309</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -826,7 +834,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>6.107969</t>
+          <t>68.376068</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -843,7 +851,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x2b58c8cc2c4a11d63f4809e837d399bdea22a0fe868c2eb6e45b6d908e34bd81</t>
+          <t>0x055ed722ad8e1fcb4f4772d6b728782e9d84139fc360e9ede36ff234eccc31e5</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -854,7 +862,7 @@
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>18.67</t>
+          <t>9.08997</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -920,7 +928,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786446437</t>
+          <t>1786447047</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -930,7 +938,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>22.359281</t>
+          <t>10.886192</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -947,27 +955,23 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x9108ebe29dd968cf40c2da378f9f378c80aa47fb35d0f66c34ba20823eac7e31</t>
+          <t>0x6f820abf55d5322626469d5a3118ee5f9c3a29d1d3a3a6a566e5b199d600f80e</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.5288</t>
+          <t>1.4863</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -975,11 +979,7 @@
           <t>Under/Over (2)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786446431</t>
+          <t>1786447020</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1042,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>1.891253</t>
+          <t>6.107969</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,39 +1059,31 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x3e490a020b088d367b2092a71abad1210bb7b27c2b51413d74ae52db826f7a65</t>
+          <t>0x2b58c8cc2c4a11d63f4809e837d399bdea22a0fe868c2eb6e45b6d908e34bd81</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>18.67</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1114,7 +1106,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1144,7 +1136,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786446420</t>
+          <t>1786446437</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1154,7 +1146,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>11.631579</t>
+          <t>22.359281</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1171,31 +1163,39 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x403efc488fdcf260a44f7bf6f00c26c8886eb1811b8c736b1a20b47ca921c66e</t>
+          <t>0x9108ebe29dd968cf40c2da378f9f378c80aa47fb35d0f66c34ba20823eac7e31</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.105</t>
+          <t>1.5288</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H8" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1248,7 +1248,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786446337</t>
+          <t>1786446431</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1258,7 +1258,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>38.952381</t>
+          <t>1.891253</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,31 +1275,39 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x531f4b82607f405ee467b383cf29c72318f248d39b819f053b24ee23023d1f70</t>
+          <t>0x3e490a020b088d367b2092a71abad1210bb7b27c2b51413d74ae52db826f7a65</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.36996</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.835</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1322,7 +1330,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1352,7 +1360,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786446336</t>
+          <t>1786446420</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1362,7 +1370,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>1.640671</t>
+          <t>11.631579</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1379,39 +1387,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0xb3a32bdd398462cad567ce66c61f991efd7fcf97116aadff293947265a593cb1</t>
+          <t>0x403efc488fdcf260a44f7bf6f00c26c8886eb1811b8c736b1a20b47ca921c66e</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>6.035</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.3912</t>
+          <t>1.105</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1434,7 +1434,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
+          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786445807</t>
+          <t>1786446337</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1474,7 +1474,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>15.42492</t>
+          <t>38.952381</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,7 +1491,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0xe14e1c541902c495d865fcecd4beaa322f341ba7d25fe03284d1ed1752b5d581</t>
+          <t>0x531f4b82607f405ee467b383cf29c72318f248d39b819f053b24ee23023d1f70</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1502,7 +1502,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.57998</t>
+          <t>1.36996</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786445791</t>
+          <t>1786446336</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1578,7 +1578,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>4.287401</t>
+          <t>1.640671</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1595,12 +1595,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0x05ff10b7369e329d09c098dea279a2087aef3f99e7333d016cc17fefdc43ac4d</t>
+          <t>0xb3a32bdd398462cad567ce66c61f991efd7fcf97116aadff293947265a593cb1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1610,22 +1610,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>27.85</t>
+          <t>6.035</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.575</t>
+          <t>1.3912</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1635,27 +1635,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1680,17 +1680,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786445438</t>
+          <t>1786445807</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>48.434783</t>
+          <t>15.42492</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,39 +1707,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0x2ec5d54c918955931d119282e1be426873e354299fd66bdf880768599903ebee</t>
+          <t>0xe14e1c541902c495d865fcecd4beaa322f341ba7d25fe03284d1ed1752b5d581</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.8513</t>
+          <t>3.57998</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.3938</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1762,7 +1754,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -1792,7 +1784,7 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786445410</t>
+          <t>1786445791</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1802,7 +1794,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>22.479492</t>
+          <t>4.287401</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1819,7 +1811,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x3d9a529160e80eb890a16c2893670e9bf2273f2addb5d0a989210dceae52707f</t>
+          <t>0x05ff10b7369e329d09c098dea279a2087aef3f99e7333d016cc17fefdc43ac4d</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1827,15 +1819,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>46.02996</t>
+          <t>27.85</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.835</t>
+          <t>1.575</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1843,7 +1839,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1851,27 +1851,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1896,17 +1896,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786445409</t>
+          <t>1786445438</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>55.125701</t>
+          <t>48.434783</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1923,31 +1923,39 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x8e51b7cdf462005f489e66cfca0c7d500669ca43fd2d3996f64b84072d635325</t>
+          <t>0x2ec5d54c918955931d119282e1be426873e354299fd66bdf880768599903ebee</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>4.27</t>
+          <t>8.8513</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.1013</t>
+          <t>1.3938</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr"/>
+          <t>Under/Over (2.5)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Over 2.5</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1970,7 +1978,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2000,7 +2008,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786445383</t>
+          <t>1786445410</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2010,7 +2018,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>42.17284</t>
+          <t>22.479492</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2027,28 +2035,28 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x56b9d5cfed219c2b12d04856ee24a476270becbad5defbb7dc7dad60a16a13a9</t>
+          <t>0x3d9a529160e80eb890a16c2893670e9bf2273f2addb5d0a989210dceae52707f</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>12.76064</t>
+          <t>46.02996</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G16" t="inlineStr"/>
@@ -2074,7 +2082,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
@@ -2104,7 +2112,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786443421</t>
+          <t>1786445409</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2114,7 +2122,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>28.919297</t>
+          <t>55.125701</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2131,23 +2139,23 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x35b58acc470365a2c9a245983b170aeeb2f01a388be1e73823eb3f0e1792d4d0</t>
+          <t>0x8e51b7cdf462005f489e66cfca0c7d500669ca43fd2d3996f64b84072d635325</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>4.27</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.1375</t>
+          <t>1.1013</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -2163,27 +2171,27 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Platense vs Coquimbo Unido</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Platense</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Coquimbo Unido</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0xb869bcff5be47e69467bcfd6e205de9f4533f12ba3b8f1bb20d9de6a5a8aec91</t>
+          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>L19052327</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
@@ -2208,17 +2216,17 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786442613</t>
+          <t>1786445383</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>1786572000</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>10.036364</t>
+          <t>42.17284</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2235,39 +2243,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
+          <t>0x56b9d5cfed219c2b12d04856ee24a476270becbad5defbb7dc7dad60a16a13a9</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>10.99999</t>
+          <t>12.76064</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2275,27 +2275,27 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
@@ -2320,17 +2320,17 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786442391</t>
+          <t>1786443421</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>18.9655</t>
+          <t>28.919297</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2347,28 +2347,28 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
+          <t>0x35b58acc470365a2c9a245983b170aeeb2f01a388be1e73823eb3f0e1792d4d0</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
       <c r="D19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.1375</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G19" t="inlineStr"/>
@@ -2379,27 +2379,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Platense vs Coquimbo Unido</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Platense</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Coquimbo Unido</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xb869bcff5be47e69467bcfd6e205de9f4533f12ba3b8f1bb20d9de6a5a8aec91</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19052327</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2424,17 +2424,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786442613</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786572000</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>23.809524</t>
+          <t>10.036364</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2451,31 +2451,39 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
+          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>27.83</t>
+          <t>10.99999</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.5825</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2498,7 +2506,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2528,7 +2536,7 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786442391</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2538,7 +2546,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>47.776824</t>
+          <t>18.9655</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2555,7 +2563,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
+          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2563,19 +2571,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>48.99946</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2583,11 +2587,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Tie</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2650,7 +2650,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>181.479481</t>
+          <t>23.809524</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2667,7 +2667,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
+          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2675,54 +2675,46 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>27.83</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.155</t>
+          <t>1.5825</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>Universidad Catolica Santiago</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
@@ -2752,7 +2744,7 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2762,7 +2754,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>12.387097</t>
+          <t>47.776824</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2779,7 +2771,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
+          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2787,15 +2779,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>48.99946</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.415</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -2803,7 +2799,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Tie</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2826,7 +2826,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2856,7 +2856,7 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>24.096386</t>
+          <t>181.479481</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2883,7 +2883,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
+          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2898,12 +2898,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>121.005</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.155</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2913,24 +2913,24 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
           <t>Estudiantes de La Plata</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
       <c r="K24" t="inlineStr">
         <is>
           <t>Universidad Catolica Santiago</t>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786440700</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>201.675</t>
+          <t>12.387097</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2995,7 +2995,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
+          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3006,12 +3006,12 @@
       <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr">
         <is>
-          <t>2.74998</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.415</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3027,27 +3027,27 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
@@ -3072,17 +3072,17 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786438265</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>3.709922</t>
+          <t>24.096386</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3099,7 +3099,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
+          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3114,12 +3114,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>19.42</t>
+          <t>121.005</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3139,27 +3139,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3184,17 +3184,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786436520</t>
+          <t>1786440700</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>34.070175</t>
+          <t>201.675</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3211,7 +3211,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
+          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3219,19 +3219,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>2.74998</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3239,26 +3235,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr">
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
       <c r="K27" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
@@ -3266,7 +3258,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3296,7 +3288,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786435951</t>
+          <t>1786438265</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3306,7 +3298,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>3.561404</t>
+          <t>3.709922</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3323,12 +3315,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
+          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3338,12 +3330,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19.42</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.1687</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -3353,32 +3345,32 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3408,7 +3400,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786435593</t>
+          <t>1786436520</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3418,7 +3410,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>266.666667</t>
+          <t>34.070175</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3435,7 +3427,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3443,15 +3435,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>90.44268</t>
+          <t>2.03</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.8363</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -3459,7 +3455,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
       <c r="H29" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786430935</t>
+          <t>1786435951</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3522,7 +3522,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>108.152682</t>
+          <t>3.561404</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3539,12 +3539,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3554,22 +3554,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>45</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.1687</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -3579,27 +3579,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Deportes Tolima vs Independiente del Valle</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Independiente del Valle</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19051703</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3624,17 +3624,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786430206</t>
+          <t>1786435593</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>1.809955</t>
+          <t>266.666667</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3651,7 +3651,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3662,17 +3662,17 @@
       <c r="C31" t="inlineStr"/>
       <c r="D31" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>90.44268</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.8363</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G31" t="inlineStr"/>
@@ -3698,7 +3698,7 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
@@ -3728,7 +3728,7 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786412670</t>
+          <t>1786430935</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -3738,7 +3738,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>108.152682</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3755,12 +3755,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3770,22 +3770,22 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.1562</t>
+          <t>1.5525</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Over 2.0</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -3795,27 +3795,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Deportes Tolima vs Independiente del Valle</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Deportes Tolima</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente del Valle</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051703</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3840,7 +3840,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786430206</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3850,7 +3850,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>1.809955</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3867,62 +3867,54 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>4.5</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.125</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I33" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
@@ -3952,7 +3944,7 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786412670</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -3962,7 +3954,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>36.0</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3979,12 +3971,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3994,22 +3986,22 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1.01</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.1562</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -4019,27 +4011,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
@@ -4064,17 +4056,17 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786395562</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>6.464</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4091,7 +4083,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -4106,22 +4098,22 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>1.8</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.18</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4146,7 +4138,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -4176,7 +4168,7 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786385932</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -4186,7 +4178,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>10.0</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4203,12 +4195,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4218,22 +4210,22 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>5.00692</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.7012</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Under/Over (1.5)</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Over 1.5</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -4258,7 +4250,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -4288,7 +4280,7 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786377754</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -4298,7 +4290,7 @@
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>7.139993</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4315,110 +4307,334 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S37" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T37" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U37" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V37" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B39" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E39" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F37" t="inlineStr">
+      <c r="F39" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr">
+      <c r="G39" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H37" t="inlineStr">
+      <c r="H39" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="I39" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J37" t="inlineStr">
+      <c r="J39" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K37" t="inlineStr">
+      <c r="K39" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
+      <c r="L39" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M37" t="inlineStr">
+      <c r="M39" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S37" t="inlineStr">
+      <c r="S39" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T37" t="inlineStr">
+      <c r="T39" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U37" t="inlineStr">
+      <c r="U39" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V37" t="inlineStr">
+      <c r="V39" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>

<commit_message>
Update soccer trades 2026-08-11 16:03:30 UTC
</commit_message>
<xml_diff>
--- a/data/sxbet/ligas/Copa Libertadores/trades.xlsx
+++ b/data/sxbet/ligas/Copa Libertadores/trades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -531,31 +531,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>0xa43e73fd0eb9b697155001cb7d168e615b053bb2384172434ebb7e2cad4f821b</t>
+          <t>0x712635a3846b3dfffbef983a3937a6a5370e5d76cfc88686bfdf33d3a18cfdf2</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>4.52999</t>
+          <t>9.2</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1.85</t>
+          <t>1.3938</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Fluminense FC -1</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -563,27 +571,27 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x4af66f5ffd6126d638275bbcb5a176772e58b9e5287cfa592c3455f80ac7d391</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
@@ -608,17 +616,17 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>1786451158</t>
+          <t>1786463878</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>5.3294</t>
+          <t>23.365079</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -635,7 +643,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>0xa379a926c9e1de27f304fc4c2c017caa09967132b53155a53855c3019d081a23</t>
+          <t>0x74818e8856c3331fdba3eba4a9b37ec931c23a8fa4c6ca3abdf75b4fa8061323</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -643,19 +651,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>7.17</t>
+          <t>179.09997</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1.56</t>
+          <t>1.84</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -663,26 +667,22 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
       <c r="K3" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
@@ -690,7 +690,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>1786450013</t>
+          <t>1786463743</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -730,7 +730,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>12.803571</t>
+          <t>213.21425</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -747,7 +747,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>0xfe9a509a313ff07389ffbf579a41acd018137e511ac3bf176d2373de751fdb99</t>
+          <t>0x734bca2c9ca76d00266785b060a16a0e1781797a99f35b4e43875e84a72eca37</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -755,23 +755,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>12.99999</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.1462</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -794,7 +802,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -824,7 +832,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>1786448309</t>
+          <t>1786463743</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -834,7 +842,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>68.376068</t>
+          <t>22.807</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -851,31 +859,39 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>0x055ed722ad8e1fcb4f4772d6b728782e9d84139fc360e9ede36ff234eccc31e5</t>
+          <t>0xc77f6ca857436bc0db9a4a360c443ad13b66422813724fcffdcca5491788b3c3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>0x97EC1C9682F70091efB04e97b0B34698cF815EE1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>9.08997</t>
+          <t>13.39</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.835</t>
+          <t>1.3938</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
+          <t>Asian Handicap (-1)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Fluminense FC -1</t>
+        </is>
+      </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -898,7 +914,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x4af66f5ffd6126d638275bbcb5a176772e58b9e5287cfa592c3455f80ac7d391</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -928,7 +944,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>1786447047</t>
+          <t>1786462194</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -938,7 +954,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>10.886192</t>
+          <t>34.006349</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -955,7 +971,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>0x6f820abf55d5322626469d5a3118ee5f9c3a29d1d3a3a6a566e5b199d600f80e</t>
+          <t>0xcb2f1253d2d1051e683579ac892fb9b825e249d53a964d120bfd31d266b08141</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -963,23 +979,31 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2.97</t>
+          <t>221.99512</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.4863</t>
+          <t>1.57</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
       <c r="H6" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1002,7 +1026,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -1032,7 +1056,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>1786447020</t>
+          <t>1786460250</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1042,7 +1066,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>6.107969</t>
+          <t>389.465123</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1059,7 +1083,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>0x2b58c8cc2c4a11d63f4809e837d399bdea22a0fe868c2eb6e45b6d908e34bd81</t>
+          <t>0xbec2a1b02b9e4febe6167741262ac4a2f4be2a5e51b0cbb57bbc5bbbbc74ec78</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -1067,15 +1091,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>18.67</t>
+          <t>26.02999</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.835</t>
+          <t>1.5637</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1083,7 +1111,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
       <c r="H7" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1106,7 +1138,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1136,7 +1168,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>1786446437</t>
+          <t>1786459213</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1146,7 +1178,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>22.359281</t>
+          <t>46.172931</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1163,12 +1195,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>0x9108ebe29dd968cf40c2da378f9f378c80aa47fb35d0f66c34ba20823eac7e31</t>
+          <t>0x5f7fb0a40c37051aca6c935ed02a8080eff54de6de82659b7b91803de699f51f</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1178,22 +1210,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8.72249</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.5288</t>
+          <t>1.3862</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Over 2.0</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1218,7 +1250,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
@@ -1248,7 +1280,7 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>1786446431</t>
+          <t>1786459213</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1258,7 +1290,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>1.891253</t>
+          <t>22.582498</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1275,12 +1307,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0x3e490a020b088d367b2092a71abad1210bb7b27c2b51413d74ae52db826f7a65</t>
+          <t>0x6980a7396690aeec170fb463350ff67029df1b9c931ec0c27ff1af059381cc58</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1290,22 +1322,22 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.21</t>
+          <t>5.79</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.19</t>
+          <t>1.3887</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Over 3.5</t>
+          <t>Fluminense FC -1</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1330,7 +1362,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x4af66f5ffd6126d638275bbcb5a176772e58b9e5287cfa592c3455f80ac7d391</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -1360,7 +1392,7 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>1786446420</t>
+          <t>1786459212</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1370,7 +1402,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>11.631579</t>
+          <t>14.893891</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -1387,7 +1419,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>0x403efc488fdcf260a44f7bf6f00c26c8886eb1811b8c736b1a20b47ca921c66e</t>
+          <t>0x112d5f4772af6b6bd83eaa569925daff03938666e745bdc007047b15ad1be063</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1398,17 +1430,17 @@
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>4.09</t>
+          <t>32.11</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.105</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -1419,27 +1451,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
@@ -1464,17 +1496,17 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>1786446337</t>
+          <t>1786454674</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>38.952381</t>
+          <t>37.776471</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -1491,7 +1523,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>0x531f4b82607f405ee467b383cf29c72318f248d39b819f053b24ee23023d1f70</t>
+          <t>0x3af4d178b0569d40395cf2b19f0b5f8a08bea2668bf4ce85dd9528580486f305</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1502,7 +1534,7 @@
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.36996</t>
+          <t>55.97</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1568,7 +1600,7 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>1786446336</t>
+          <t>1786454672</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1578,7 +1610,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>1.640671</t>
+          <t>67.02994</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -1595,12 +1627,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>0xb3a32bdd398462cad567ce66c61f991efd7fcf97116aadff293947265a593cb1</t>
+          <t>0xa4db1189dcf9cf5de113c29d278457074a70fb41495314c3d482543503c28879</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1610,22 +1642,22 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6.035</t>
+          <t>36.98</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.3912</t>
+          <t>1.575</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Over 2.5</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1635,27 +1667,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
@@ -1680,17 +1712,17 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>1786445807</t>
+          <t>1786454526</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>15.42492</t>
+          <t>64.313043</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
@@ -1707,23 +1739,23 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>0xe14e1c541902c495d865fcecd4beaa322f341ba7d25fe03284d1ed1752b5d581</t>
+          <t>0xa43e73fd0eb9b697155001cb7d168e615b053bb2384172434ebb7e2cad4f821b</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3.57998</t>
+          <t>4.52999</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.835</t>
+          <t>1.85</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1739,27 +1771,27 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
@@ -1784,17 +1816,17 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>1786445791</t>
+          <t>1786451158</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>4.287401</t>
+          <t>5.3294</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
@@ -1811,7 +1843,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>0x05ff10b7369e329d09c098dea279a2087aef3f99e7333d016cc17fefdc43ac4d</t>
+          <t>0xa379a926c9e1de27f304fc4c2c017caa09967132b53155a53855c3019d081a23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1826,12 +1858,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>27.85</t>
+          <t>7.17</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>1.575</t>
+          <t>1.56</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1841,7 +1873,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1851,27 +1883,27 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
@@ -1896,17 +1928,17 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>1786445438</t>
+          <t>1786450013</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>48.434783</t>
+          <t>12.803571</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
@@ -1923,39 +1955,31 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>0x2ec5d54c918955931d119282e1be426873e354299fd66bdf880768599903ebee</t>
+          <t>0xfe9a509a313ff07389ffbf579a41acd018137e511ac3bf176d2373de751fdb99</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
       <c r="D15" t="inlineStr">
         <is>
-          <t>8.8513</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1.3938</t>
+          <t>1.1462</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Under/Over (2.5)</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Over 2.5</t>
-        </is>
-      </c>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -1978,7 +2002,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
@@ -2008,7 +2032,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>1786445410</t>
+          <t>1786448309</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2018,7 +2042,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>22.479492</t>
+          <t>68.376068</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
@@ -2035,7 +2059,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>0x3d9a529160e80eb890a16c2893670e9bf2273f2addb5d0a989210dceae52707f</t>
+          <t>0x055ed722ad8e1fcb4f4772d6b728782e9d84139fc360e9ede36ff234eccc31e5</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2046,7 +2070,7 @@
       <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr">
         <is>
-          <t>46.02996</t>
+          <t>9.08997</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -2112,7 +2136,7 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>1786445409</t>
+          <t>1786447047</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2122,7 +2146,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>55.125701</t>
+          <t>10.886192</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
@@ -2139,7 +2163,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>0x8e51b7cdf462005f489e66cfca0c7d500669ca43fd2d3996f64b84072d635325</t>
+          <t>0x6f820abf55d5322626469d5a3118ee5f9c3a29d1d3a3a6a566e5b199d600f80e</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -2150,17 +2174,17 @@
       <c r="C17" t="inlineStr"/>
       <c r="D17" t="inlineStr">
         <is>
-          <t>4.27</t>
+          <t>2.97</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.1013</t>
+          <t>1.4863</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
+          <t>Under/Over (2)</t>
         </is>
       </c>
       <c r="G17" t="inlineStr"/>
@@ -2186,7 +2210,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2216,7 +2240,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>1786445383</t>
+          <t>1786447020</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2226,7 +2250,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>42.17284</t>
+          <t>6.107969</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2243,28 +2267,28 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>0x56b9d5cfed219c2b12d04856ee24a476270becbad5defbb7dc7dad60a16a13a9</t>
+          <t>0x2b58c8cc2c4a11d63f4809e837d399bdea22a0fe868c2eb6e45b6d908e34bd81</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>12.76064</t>
+          <t>18.67</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.4412</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G18" t="inlineStr"/>
@@ -2290,7 +2314,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
@@ -2320,7 +2344,7 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>1786443421</t>
+          <t>1786446437</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2330,7 +2354,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>28.919297</t>
+          <t>22.359281</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
@@ -2347,31 +2371,39 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>0x35b58acc470365a2c9a245983b170aeeb2f01a388be1e73823eb3f0e1792d4d0</t>
+          <t>0x9108ebe29dd968cf40c2da378f9f378c80aa47fb35d0f66c34ba20823eac7e31</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.38</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.1375</t>
+          <t>1.5288</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under/Over (0.5)</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr"/>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2379,27 +2411,27 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Platense vs Coquimbo Unido</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Platense</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Coquimbo Unido</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0xb869bcff5be47e69467bcfd6e205de9f4533f12ba3b8f1bb20d9de6a5a8aec91</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>L19052327</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
@@ -2424,17 +2456,17 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>1786442613</t>
+          <t>1786446431</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>1786572000</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>10.036364</t>
+          <t>1.891253</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
@@ -2451,12 +2483,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
+          <t>0x3e490a020b088d367b2092a71abad1210bb7b27c2b51413d74ae52db826f7a65</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2466,22 +2498,22 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>10.99999</t>
+          <t>2.21</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.58</t>
+          <t>1.19</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (3.5)</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Over 3.5</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -2491,27 +2523,27 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
@@ -2536,17 +2568,17 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>1786442391</t>
+          <t>1786446420</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>18.9655</t>
+          <t>11.631579</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
@@ -2563,7 +2595,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
+          <t>0x403efc488fdcf260a44f7bf6f00c26c8886eb1811b8c736b1a20b47ca921c66e</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2574,17 +2606,17 @@
       <c r="C21" t="inlineStr"/>
       <c r="D21" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>4.09</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.42</t>
+          <t>1.105</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (0.5)</t>
         </is>
       </c>
       <c r="G21" t="inlineStr"/>
@@ -2595,27 +2627,27 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
@@ -2640,17 +2672,17 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786446337</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>23.809524</t>
+          <t>38.952381</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
@@ -2667,7 +2699,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
+          <t>0x531f4b82607f405ee467b383cf29c72318f248d39b819f053b24ee23023d1f70</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2678,17 +2710,17 @@
       <c r="C22" t="inlineStr"/>
       <c r="D22" t="inlineStr">
         <is>
-          <t>27.83</t>
+          <t>1.36996</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.5825</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Asian Handicap (-1)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G22" t="inlineStr"/>
@@ -2699,27 +2731,27 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
@@ -2744,17 +2776,17 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786446336</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>47.776824</t>
+          <t>1.640671</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2771,12 +2803,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
+          <t>0xb3a32bdd398462cad567ce66c61f991efd7fcf97116aadff293947265a593cb1</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2786,22 +2818,22 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>48.99946</t>
+          <t>6.035</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.27</t>
+          <t>1.3912</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Tie</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2811,27 +2843,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
@@ -2856,17 +2888,17 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>1786441819</t>
+          <t>1786445807</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>181.479481</t>
+          <t>15.42492</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
@@ -2883,7 +2915,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
+          <t>0xe14e1c541902c495d865fcecd4beaa322f341ba7d25fe03284d1ed1752b5d581</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2891,19 +2923,15 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C24" t="inlineStr"/>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.92</t>
+          <t>3.57998</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.155</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -2911,11 +2939,7 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
+      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -2923,27 +2947,27 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
@@ -2968,17 +2992,17 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786445791</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>12.387097</t>
+          <t>4.287401</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
@@ -2995,7 +3019,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
+          <t>0x05ff10b7369e329d09c098dea279a2087aef3f99e7333d016cc17fefdc43ac4d</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3003,15 +3027,19 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>27.85</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.415</t>
+          <t>1.575</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3019,7 +3047,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H25" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -3072,7 +3104,7 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>1786441818</t>
+          <t>1786445438</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -3082,7 +3114,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>24.096386</t>
+          <t>48.434783</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
@@ -3099,12 +3131,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
+          <t>0x2ec5d54c918955931d119282e1be426873e354299fd66bdf880768599903ebee</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+          <t>0x40C6406af6250bDC2d12E0AA4053630789f332c2</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3114,22 +3146,22 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>121.005</t>
+          <t>8.8513</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1.6</t>
+          <t>1.3938</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>1X2</t>
+          <t>Under/Over (2.5)</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Over 2.5</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -3139,27 +3171,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Estudiantes de La Plata</t>
+          <t>Fluminense FC</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Universidad Catolica Santiago</t>
+          <t>Independiente Rivadavia</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
+          <t>0xef18e00af5377adf650979c43f65d316f868149306345fc917c36209c9ddbbc5</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>L19052123</t>
+          <t>L19051697</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
@@ -3184,17 +3216,17 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>1786440700</t>
+          <t>1786445410</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>1786494600</t>
+          <t>1786485600</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>201.675</t>
+          <t>22.479492</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
@@ -3211,7 +3243,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
+          <t>0x3d9a529160e80eb890a16c2893670e9bf2273f2addb5d0a989210dceae52707f</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3222,12 +3254,12 @@
       <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr">
         <is>
-          <t>2.74998</t>
+          <t>46.02996</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1.7412</t>
+          <t>1.835</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -3258,7 +3290,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
@@ -3288,7 +3320,7 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>1786438265</t>
+          <t>1786445409</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -3298,7 +3330,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>3.709922</t>
+          <t>55.125701</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
@@ -3315,7 +3347,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
+          <t>0x8e51b7cdf462005f489e66cfca0c7d500669ca43fd2d3996f64b84072d635325</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3323,46 +3355,38 @@
           <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+      <c r="C28" t="inlineStr"/>
       <c r="D28" t="inlineStr">
         <is>
-          <t>19.42</t>
+          <t>4.27</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.1013</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
       <c r="K28" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
@@ -3370,7 +3394,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x80d8175828dec9206ae65dc5ec03e79fe468294b0bcce7531d8faeccee6c8f1a</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
@@ -3400,7 +3424,7 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>1786436520</t>
+          <t>1786445383</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -3410,7 +3434,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>34.070175</t>
+          <t>42.17284</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
@@ -3427,54 +3451,46 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
+          <t>0x56b9d5cfed219c2b12d04856ee24a476270becbad5defbb7dc7dad60a16a13a9</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xa141274f45d09C2533035cd3c6ab42F3470dF7A8</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr"/>
       <c r="D29" t="inlineStr">
         <is>
-          <t>2.03</t>
+          <t>12.76064</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.57</t>
+          <t>1.4412</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>Fluminense FC</t>
-        </is>
-      </c>
       <c r="K29" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
@@ -3482,7 +3498,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+          <t>0x39394bc5d9cfce03d8a121f78750dd20929641d0f65b038d3d3fca4decabf306</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
@@ -3512,7 +3528,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>1786435951</t>
+          <t>1786443421</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3522,7 +3538,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>3.561404</t>
+          <t>28.919297</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
@@ -3539,39 +3555,31 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
+          <t>0x35b58acc470365a2c9a245983b170aeeb2f01a388be1e73823eb3f0e1792d4d0</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr"/>
       <c r="D30" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>1.38</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.1687</t>
+          <t>1.1375</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>1X2</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>Independiente Rivadavia</t>
-        </is>
-      </c>
+          <t>Under/Over (0.5)</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -3579,27 +3587,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Platense vs Coquimbo Unido</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Platense</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Coquimbo Unido</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0xb869bcff5be47e69467bcfd6e205de9f4533f12ba3b8f1bb20d9de6a5a8aec91</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052327</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
@@ -3624,17 +3632,17 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>1786435593</t>
+          <t>1786442613</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786572000</t>
         </is>
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>266.666667</t>
+          <t>10.036364</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
@@ -3651,23 +3659,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+          <t>0x1a004f4096e99abbb184b28187ee805db67cbf756edee0d02846ee7c440fdfb6</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr"/>
+          <t>0xBc04c6a7E9255Cb262632407a40Aa6344137555b</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>90.44268</t>
+          <t>10.99999</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.8363</t>
+          <t>1.58</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -3675,7 +3687,11 @@
           <t>1X2</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
       <c r="H31" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -3683,27 +3699,27 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
@@ -3728,17 +3744,17 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>1786430935</t>
+          <t>1786442391</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>108.152682</t>
+          <t>18.9655</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
@@ -3755,39 +3771,31 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+          <t>0xc31a2d511f507028887b35c0973e47baf1f105ef2e95f25e4b74805f03f66b63</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr"/>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.5525</t>
+          <t>1.42</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Under/Over (2)</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>Over 2.0</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -3795,27 +3803,27 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Deportes Tolima vs Independiente del Valle</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Deportes Tolima</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Independiente del Valle</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>L19051703</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
@@ -3840,7 +3848,7 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>1786430206</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -3850,7 +3858,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>1.809955</t>
+          <t>23.809524</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
@@ -3867,7 +3875,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+          <t>0x99825dfd289068cfc87e04222379f1f4cffacb4baf5a72fe751a2fa1a61f4073</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3878,17 +3886,17 @@
       <c r="C33" t="inlineStr"/>
       <c r="D33" t="inlineStr">
         <is>
-          <t>4.5</t>
+          <t>27.83</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.5825</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Under/Over (1)</t>
+          <t>Asian Handicap (-1)</t>
         </is>
       </c>
       <c r="G33" t="inlineStr"/>
@@ -3899,27 +3907,27 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+          <t>0x14691c65ea5d066fdde5e3cacc8b9b24f5292a9a387a4f7823d98c5f0a120af2</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
@@ -3944,17 +3952,17 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>1786412670</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>36.0</t>
+          <t>47.776824</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
@@ -3971,12 +3979,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+          <t>0x89efaad177a4126944b3f2110f71e592394cc4d9e91052ab3fdf330485fd9c87</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3986,12 +3994,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.01</t>
+          <t>48.99946</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.1562</t>
+          <t>1.27</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -4001,32 +4009,32 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
+          <t>Tie</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
           <t>Universidad Catolica Santiago</t>
         </is>
       </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Copa Libertadores</t>
-        </is>
-      </c>
-      <c r="I34" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>Estudiantes de La Plata</t>
-        </is>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>Universidad Catolica Santiago</t>
-        </is>
-      </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+          <t>0x39a4427bf391b117de6321de7c25d17c15f7a5ef0fe564e928ff746df913bd11</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
@@ -4056,7 +4064,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>1786395562</t>
+          <t>1786441819</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -4066,7 +4074,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>6.464</t>
+          <t>181.479481</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
@@ -4083,12 +4091,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+          <t>0xa4fd915db15f8490552ed36816875192e70cc52e0206178c1e4bae900ec7d228</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4098,12 +4106,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.8</t>
+          <t>1.92</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.18</t>
+          <t>1.155</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -4113,7 +4121,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4123,27 +4131,27 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
@@ -4168,17 +4176,17 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>1786385932</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>10.0</t>
+          <t>12.387097</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
@@ -4195,39 +4203,31 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+          <t>0x8fc2706f7995ba1a805ba3fc8c58db55cf56ca3a37cb162a0722fc4f8cb6b6c1</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
       <c r="D36" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.415</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>Over 1.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -4235,27 +4235,27 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
@@ -4280,17 +4280,17 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>1786377754</t>
+          <t>1786441818</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>24.096386</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
@@ -4307,12 +4307,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+          <t>0x2eb767983653bc696ef93825f3e57f7762e13853f64c8f856b8e6a5ec149157e</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4322,22 +4322,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>5.00692</t>
+          <t>121.005</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.7012</t>
+          <t>1.6</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Under/Over (1.5)</t>
+          <t>1X2</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Over 1.5</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -4347,27 +4347,27 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Fluminense FC vs Independiente Rivadavia</t>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Fluminense FC</t>
+          <t>Estudiantes de La Plata</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Independiente Rivadavia</t>
+          <t>Universidad Catolica Santiago</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+          <t>0x4dc78bb6be3462cd1fab24e2b0da51d5b57ba97aa20026605473e7813d0def66</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>L19051697</t>
+          <t>L19052123</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
@@ -4392,17 +4392,17 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>1786377751</t>
+          <t>1786440700</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>1786485600</t>
+          <t>1786494600</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>7.139993</t>
+          <t>201.675</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
@@ -4419,39 +4419,31 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+          <t>0x29a00adde01bfc415a64526402912b920363d439a6884efd0cb43a770598e8a0</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2.27</t>
+          <t>2.74998</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>1.2263</t>
+          <t>1.7412</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Under/Over (3.5)</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>Over 3.5</t>
-        </is>
-      </c>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
@@ -4474,7 +4466,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+          <t>0x92508bdbb50200c3f9ccf48a035fe626c5258657b158e0da0b6d5676e031561c</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -4504,7 +4496,7 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>1786369612</t>
+          <t>1786438265</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
@@ -4514,7 +4506,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>10.033149</t>
+          <t>3.709922</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
@@ -4531,110 +4523,1326 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>0x319d834586df2cf39f21f64782e56531a38b492cb515c0857c1eaf394d718c34</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>19.42</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>1786436520</t>
+        </is>
+      </c>
+      <c r="S39" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T39" t="inlineStr">
+        <is>
+          <t>34.070175</t>
+        </is>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V39" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>0x96b6c83684ff1720d43571152f25177b097a58db1786aebd3907582d4e7f904d</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>2.03</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>1.57</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>0x94f6c751ba8b0174e4f18d10eb88eb44da9655f4f60abb5bd3dc71922f0c6e25</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>1786435951</t>
+        </is>
+      </c>
+      <c r="S40" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T40" t="inlineStr">
+        <is>
+          <t>3.561404</t>
+        </is>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>0x0b3f2c5896b46063d7824afecc68425c611033d6e110bf65f74b44e42cbf563f</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>0x68E1818FF20BBe84F9be9E0A4A395FB11079Bd35</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>1.1687</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>1786435593</t>
+        </is>
+      </c>
+      <c r="S41" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T41" t="inlineStr">
+        <is>
+          <t>266.666667</t>
+        </is>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>0xbcf048a881cdf1035f22f93a76d9c2d8ee1cbc73d409e86459bce8b623e8c866</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>90.44268</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>1.8363</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>1786430935</t>
+        </is>
+      </c>
+      <c r="S42" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T42" t="inlineStr">
+        <is>
+          <t>108.152682</t>
+        </is>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>0xbe724ec46774277cf53d6a48cf08ae67871536f45a8d35b673483bd5d7224274</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>0x5D69C3af95Ff47088b415B25F41b1fFDc8571063</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>1.5525</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Under/Over (2)</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Over 2.0</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Deportes Tolima vs Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Deportes Tolima</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Independiente del Valle</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>0x2d0bac9df7c6a154b43afbe4b7422080dd88aa1a0304c173a96568f3bd111299</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>L19051703</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr">
+        <is>
+          <t>1786430206</t>
+        </is>
+      </c>
+      <c r="S43" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T43" t="inlineStr">
+        <is>
+          <t>1.809955</t>
+        </is>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>0xc890b61f7f040a88f9534757b2d3679b6d83d3408dbd284fc67e9933bc55e728</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>0xFD3a22179CA4104E97c670b834750Bd7Ff310b17</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>1.125</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Under/Over (1)</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>0x4de4f6a4237fd766197c4b0afb35539dfd5602f132ebd57d54ec46c416de5d44</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr">
+        <is>
+          <t>1786412670</t>
+        </is>
+      </c>
+      <c r="S44" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T44" t="inlineStr">
+        <is>
+          <t>36.0</t>
+        </is>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>0x174a2c32c747fefccf5c826d99065ff5c5732ab578abb22dccb1f974effcdbde</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>1.01</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>1.1562</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata vs Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Estudiantes de La Plata</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Universidad Catolica Santiago</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>0xce4ecd8dd623e1b5a12a5eb01e2d45f95e3055333367cfd5fda32e73c5330e61</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>L19052123</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr">
+        <is>
+          <t>1786395562</t>
+        </is>
+      </c>
+      <c r="S45" t="inlineStr">
+        <is>
+          <t>1786494600</t>
+        </is>
+      </c>
+      <c r="T45" t="inlineStr">
+        <is>
+          <t>6.464</t>
+        </is>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>0x698e92b969ccfad587b8ec954671b5328cdce0487a25e27544c610ebb082f2b7</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>1.18</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1X2</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>0xb0ffbe65243cad0ebe3452ebe89494ff47978b8594f9aaeecb17c126c2dad6a2</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr">
+        <is>
+          <t>1786385932</t>
+        </is>
+      </c>
+      <c r="S46" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T46" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>0xe5c4a369af4933ac468142f4356efc72283a57c47ec6352d2c4b65e2ea27e80b</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>1786377754</t>
+        </is>
+      </c>
+      <c r="S47" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T47" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>0x23802563416b16627a0721f8adf02a15e37b1269ba8ecd89e62101af682142e2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>0x3b2B3900de9f93d1a397Efd858D1035643D15F96</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>5.00692</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>1.7012</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Under/Over (1.5)</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Over 1.5</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr">
+        <is>
+          <t>1786377751</t>
+        </is>
+      </c>
+      <c r="S48" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T48" t="inlineStr">
+        <is>
+          <t>7.139993</t>
+        </is>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>0xbbe4f298e1d19f20fabc50aeaa116d34e372b93e0f601f20d348cf673b9b251b</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>2.27</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>1.2263</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Under/Over (3.5)</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Over 3.5</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>Copa Libertadores</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>Fluminense FC vs Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Fluminense FC</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Independiente Rivadavia</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>0xc21158e40ca0c03ab3a5b699371a3473d9bfbb38e46c828c2d565753cf9ec148</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>L19051697</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr">
+        <is>
+          <t>SUCCESS</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr">
+        <is>
+          <t>1786369612</t>
+        </is>
+      </c>
+      <c r="S49" t="inlineStr">
+        <is>
+          <t>1786485600</t>
+        </is>
+      </c>
+      <c r="T49" t="inlineStr">
+        <is>
+          <t>10.033149</t>
+        </is>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>SXR</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
           <t>0x831aaf6a20d39c81af2877439ef96d74f91cde472d0e0657c78f797db64dbb8f</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>0x740d5718a79A8559fEeE8B00922F8Cd773A81D84</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
         <is>
           <t>8.24</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>1.6975</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F50" t="inlineStr">
         <is>
           <t>Under/Over (1.5)</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G50" t="inlineStr">
         <is>
           <t>Over 1.5</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
+      <c r="H50" t="inlineStr">
         <is>
           <t>Copa Libertadores</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="I50" t="inlineStr">
         <is>
           <t>Fluminense FC vs Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="J39" t="inlineStr">
+      <c r="J50" t="inlineStr">
         <is>
           <t>Fluminense FC</t>
         </is>
       </c>
-      <c r="K39" t="inlineStr">
+      <c r="K50" t="inlineStr">
         <is>
           <t>Independiente Rivadavia</t>
         </is>
       </c>
-      <c r="L39" t="inlineStr">
+      <c r="L50" t="inlineStr">
         <is>
           <t>0x78244709b8d787ac24e9571b80b4dfd06844796fe736fb554c5121edd298aec5</t>
         </is>
       </c>
-      <c r="M39" t="inlineStr">
+      <c r="M50" t="inlineStr">
         <is>
           <t>L19051697</t>
         </is>
       </c>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr">
         <is>
           <t>SUCCESS</t>
         </is>
       </c>
-      <c r="Q39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="R39" t="inlineStr">
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr">
         <is>
           <t>1786333027</t>
         </is>
       </c>
-      <c r="S39" t="inlineStr">
+      <c r="S50" t="inlineStr">
         <is>
           <t>1786485600</t>
         </is>
       </c>
-      <c r="T39" t="inlineStr">
+      <c r="T50" t="inlineStr">
         <is>
           <t>11.81362</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="U50" t="inlineStr">
         <is>
           <t>SXR</t>
         </is>
       </c>
-      <c r="V39" t="inlineStr">
+      <c r="V50" t="inlineStr">
         <is>
           <t>0x6629Ce1Cf35Cc1329ebB4F63202F3f197b3F050B</t>
         </is>

</xml_diff>